<commit_message>
modifies code to combine SDZWA metadata differently (all in R). Modifies code to work up the plots for the hormone and DNA extraction methods paper
</commit_message>
<xml_diff>
--- a/metadata/Plate2/SRKW_Diet_Plate2_MetaData.xlsx
+++ b/metadata/Plate2/SRKW_Diet_Plate2_MetaData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lfallon/Library/Application Support/Box/Box Edit/Documents/2185572405481/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/mball3_uw_edu/Documents/Documents/WADE LAB/SRKW/metadata/Plate2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="160" documentId="13_ncr:1_{E2D37667-AD52-244F-8552-D2CF91E538CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AAE051D-0BD5-41C5-94C5-4B0DE8AB882D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348E722D-DFD7-8D47-9A75-F23C3A7DC44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6200" yWindow="680" windowWidth="20580" windowHeight="22820" xr2:uid="{518B7A33-C5FE-E642-B8D5-47A99A98280E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{518B7A33-C5FE-E642-B8D5-47A99A98280E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="79">
   <si>
     <t>Sample_no</t>
   </si>
@@ -240,13 +240,46 @@
   </si>
   <si>
     <t>F23JUL03.03A-Lys</t>
+  </si>
+  <si>
+    <t>J51</t>
+  </si>
+  <si>
+    <t>J26</t>
+  </si>
+  <si>
+    <t>J57</t>
+  </si>
+  <si>
+    <t>L121</t>
+  </si>
+  <si>
+    <t>J49</t>
+  </si>
+  <si>
+    <t>J41</t>
+  </si>
+  <si>
+    <t>J56</t>
+  </si>
+  <si>
+    <t>J27</t>
+  </si>
+  <si>
+    <t>J39</t>
+  </si>
+  <si>
+    <t>K33</t>
+  </si>
+  <si>
+    <t>K12</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -289,19 +322,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -639,13 +669,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A0E5F67-981F-2842-8BC9-09C804A53EC3}">
   <dimension ref="A1:G70"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="2" max="2" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.875" customWidth="1"/>
+    <col min="2" max="2" width="22.8125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.8125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -668,7 +698,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -688,7 +718,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -708,13 +738,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
+      <c r="D4" t="s">
+        <v>68</v>
+      </c>
       <c r="E4">
         <v>2022</v>
       </c>
@@ -725,7 +758,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -745,13 +778,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
+      <c r="D6" t="s">
+        <v>57</v>
+      </c>
       <c r="E6">
         <v>2025</v>
       </c>
@@ -762,13 +798,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>18</v>
       </c>
+      <c r="D7" t="s">
+        <v>57</v>
+      </c>
       <c r="E7">
         <v>2025</v>
       </c>
@@ -779,13 +818,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
       </c>
+      <c r="D8" t="s">
+        <v>69</v>
+      </c>
       <c r="E8">
         <v>2025</v>
       </c>
@@ -796,13 +838,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
+      <c r="D9" t="s">
+        <v>70</v>
+      </c>
       <c r="E9">
         <v>2025</v>
       </c>
@@ -813,13 +858,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>21</v>
       </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
       <c r="E10">
         <v>2025</v>
       </c>
@@ -830,13 +878,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>22</v>
       </c>
+      <c r="D11" t="s">
+        <v>69</v>
+      </c>
       <c r="E11">
         <v>2018</v>
       </c>
@@ -847,13 +898,16 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>23</v>
       </c>
+      <c r="D12" t="s">
+        <v>69</v>
+      </c>
       <c r="E12">
         <v>2018</v>
       </c>
@@ -864,13 +918,16 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>24</v>
       </c>
+      <c r="D13" t="s">
+        <v>71</v>
+      </c>
       <c r="E13">
         <v>2022</v>
       </c>
@@ -881,13 +938,16 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>25</v>
       </c>
+      <c r="D14" t="s">
+        <v>72</v>
+      </c>
       <c r="E14">
         <v>2023</v>
       </c>
@@ -898,13 +958,16 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
       </c>
+      <c r="D15" t="s">
+        <v>73</v>
+      </c>
       <c r="E15">
         <v>2025</v>
       </c>
@@ -915,13 +978,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>28</v>
       </c>
+      <c r="D16" t="s">
+        <v>8</v>
+      </c>
       <c r="E16">
         <v>2025</v>
       </c>
@@ -932,7 +998,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -942,6 +1008,9 @@
       <c r="C17" t="s">
         <v>30</v>
       </c>
+      <c r="D17" t="s">
+        <v>8</v>
+      </c>
       <c r="E17">
         <v>2025</v>
       </c>
@@ -952,7 +1021,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -962,6 +1031,9 @@
       <c r="C18" t="s">
         <v>32</v>
       </c>
+      <c r="D18" t="s">
+        <v>8</v>
+      </c>
       <c r="E18">
         <v>2025</v>
       </c>
@@ -972,13 +1044,16 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>33</v>
       </c>
+      <c r="D19" t="s">
+        <v>74</v>
+      </c>
       <c r="E19">
         <v>2025</v>
       </c>
@@ -989,13 +1064,16 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>35</v>
       </c>
+      <c r="D20" t="s">
+        <v>74</v>
+      </c>
       <c r="E20">
         <v>2025</v>
       </c>
@@ -1006,7 +1084,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1016,6 +1094,9 @@
       <c r="C21" t="s">
         <v>30</v>
       </c>
+      <c r="D21" t="s">
+        <v>74</v>
+      </c>
       <c r="E21">
         <v>2025</v>
       </c>
@@ -1026,7 +1107,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1036,6 +1117,9 @@
       <c r="C22" t="s">
         <v>32</v>
       </c>
+      <c r="D22" t="s">
+        <v>74</v>
+      </c>
       <c r="E22">
         <v>2025</v>
       </c>
@@ -1046,13 +1130,16 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>38</v>
       </c>
+      <c r="D23" t="s">
+        <v>75</v>
+      </c>
       <c r="E23">
         <v>2025</v>
       </c>
@@ -1063,13 +1150,16 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
         <v>39</v>
       </c>
+      <c r="D24" t="s">
+        <v>75</v>
+      </c>
       <c r="E24">
         <v>2025</v>
       </c>
@@ -1080,13 +1170,16 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
         <v>40</v>
       </c>
+      <c r="D25" t="s">
+        <v>8</v>
+      </c>
       <c r="E25">
         <v>2025</v>
       </c>
@@ -1097,7 +1190,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1107,6 +1200,9 @@
       <c r="C26" t="s">
         <v>30</v>
       </c>
+      <c r="D26" t="s">
+        <v>76</v>
+      </c>
       <c r="E26">
         <v>2025</v>
       </c>
@@ -1117,7 +1213,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1127,6 +1223,9 @@
       <c r="C27" t="s">
         <v>32</v>
       </c>
+      <c r="D27" t="s">
+        <v>76</v>
+      </c>
       <c r="E27">
         <v>2025</v>
       </c>
@@ -1137,13 +1236,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
         <v>43</v>
       </c>
+      <c r="D28" t="s">
+        <v>69</v>
+      </c>
       <c r="E28">
         <v>2025</v>
       </c>
@@ -1154,7 +1256,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1171,13 +1273,16 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
         <v>45</v>
       </c>
+      <c r="D30" t="s">
+        <v>46</v>
+      </c>
       <c r="E30" s="3" t="s">
         <v>46</v>
       </c>
@@ -1188,13 +1293,16 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
         <v>47</v>
       </c>
+      <c r="D31" t="s">
+        <v>72</v>
+      </c>
       <c r="E31">
         <v>2025</v>
       </c>
@@ -1205,13 +1313,16 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
         <v>48</v>
       </c>
+      <c r="D32" t="s">
+        <v>74</v>
+      </c>
       <c r="E32">
         <v>2025</v>
       </c>
@@ -1222,13 +1333,16 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
         <v>49</v>
       </c>
+      <c r="D33" t="s">
+        <v>77</v>
+      </c>
       <c r="E33">
         <v>2025</v>
       </c>
@@ -1239,13 +1353,16 @@
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
         <v>51</v>
       </c>
+      <c r="D34" t="s">
+        <v>78</v>
+      </c>
       <c r="E34">
         <v>2026</v>
       </c>
@@ -1256,13 +1373,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
         <v>53</v>
       </c>
+      <c r="D35" t="s">
+        <v>57</v>
+      </c>
       <c r="E35">
         <v>2026</v>
       </c>
@@ -1273,7 +1393,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1283,6 +1403,9 @@
       <c r="C36" t="s">
         <v>30</v>
       </c>
+      <c r="D36" t="s">
+        <v>70</v>
+      </c>
       <c r="E36">
         <v>2026</v>
       </c>
@@ -1293,7 +1416,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1303,6 +1426,9 @@
       <c r="C37" t="s">
         <v>32</v>
       </c>
+      <c r="D37" t="s">
+        <v>70</v>
+      </c>
       <c r="E37">
         <v>2026</v>
       </c>
@@ -1313,7 +1439,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1333,14 +1459,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
         <v>58</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E39">
@@ -1353,7 +1479,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1373,7 +1499,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1393,7 +1519,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1413,13 +1539,16 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
         <v>66</v>
       </c>
+      <c r="D43" t="s">
+        <v>16</v>
+      </c>
       <c r="E43">
         <v>2023</v>
       </c>
@@ -1430,7 +1559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1447,38 +1576,38 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:7"/>
-    <row r="46" spans="1:7"/>
-    <row r="47" spans="1:7"/>
-    <row r="48" spans="1:7"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65" spans="5:7"/>
-    <row r="66" spans="5:7"/>
-    <row r="67" spans="5:7"/>
-    <row r="68" spans="5:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.5"/>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.5"/>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.5"/>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.5"/>
+    <row r="49" x14ac:dyDescent="0.5"/>
+    <row r="50" x14ac:dyDescent="0.5"/>
+    <row r="51" x14ac:dyDescent="0.5"/>
+    <row r="52" x14ac:dyDescent="0.5"/>
+    <row r="53" x14ac:dyDescent="0.5"/>
+    <row r="54" x14ac:dyDescent="0.5"/>
+    <row r="55" x14ac:dyDescent="0.5"/>
+    <row r="56" x14ac:dyDescent="0.5"/>
+    <row r="57" x14ac:dyDescent="0.5"/>
+    <row r="58" x14ac:dyDescent="0.5"/>
+    <row r="59" x14ac:dyDescent="0.5"/>
+    <row r="60" x14ac:dyDescent="0.5"/>
+    <row r="61" x14ac:dyDescent="0.5"/>
+    <row r="62" x14ac:dyDescent="0.5"/>
+    <row r="63" x14ac:dyDescent="0.5"/>
+    <row r="64" x14ac:dyDescent="0.5"/>
+    <row r="65" spans="5:7" x14ac:dyDescent="0.5"/>
+    <row r="66" spans="5:7" x14ac:dyDescent="0.5"/>
+    <row r="67" spans="5:7" x14ac:dyDescent="0.5"/>
+    <row r="68" spans="5:7" x14ac:dyDescent="0.5">
       <c r="E68" s="1"/>
       <c r="G68" s="1"/>
     </row>
-    <row r="69" spans="5:7">
+    <row r="69" spans="5:7" x14ac:dyDescent="0.5">
       <c r="E69" s="1"/>
       <c r="G69" s="1"/>
     </row>
-    <row r="70" spans="5:7">
+    <row r="70" spans="5:7" x14ac:dyDescent="0.5">
       <c r="E70" s="1"/>
     </row>
   </sheetData>

</xml_diff>